<commit_message>
feat(payments): read the Commentaire column of the payments export
- Added `Line.Comment`, read from the optional « Commentaire » column by `findColumns` and `readLine`; lines stored before read back with an empty comment.
- Left the column out of `MissingColumns`: an export without it only lacks the comments.
- Replaced the comment witness of the fixtures with `fixtureComment` on the Levant line, still absent from the database file in clear.
- Regenerated `payments_valid.xlsx` and updated the README's list of what the service reads.
</commit_message>
<xml_diff>
--- a/testdata/fixtures/payments_missing_column.xlsx
+++ b/testdata/fixtures/payments_missing_column.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t xml:space="preserve">Nom</t>
   </si>
@@ -95,9 +95,6 @@
   </si>
   <si>
     <t xml:space="preserve">Détendeur et gilet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commentaire privé du paiement</t>
   </si>
   <si>
     <t xml:space="preserve">Mme</t>
@@ -225,23 +222,20 @@
       <c r="O2" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>29</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>30</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>31</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>32</v>
       </c>
-      <c r="U2" t="s">
+      <c r="X2" t="s">
         <v>33</v>
-      </c>
-      <c r="X2" t="s">
-        <v>34</v>
       </c>
       <c r="Y2">
         <v>0</v>

</xml_diff>